<commit_message>
until index 7 of economic working
</commit_message>
<xml_diff>
--- a/outputs/views_single_sheet.xlsx
+++ b/outputs/views_single_sheet.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="demographics" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="tourism" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="economics" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9494,4 +9495,1823 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:BI60"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>consumer_confidence_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>geo</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2021-01</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2021-02</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2021-03</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2021-04</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2021-05</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2021-06</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2021-07</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2021-08</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2021-09</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2021-10</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2021-11</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2021-12</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>2022-01</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>2022-02</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>2022-03</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>2022-04</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>2022-05</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>2022-06</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>2022-07</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>2022-08</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>2022-09</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>2022-10</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>2022-11</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>2022-12</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>2023-01</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>2023-02</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>2023-03</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>2023-04</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>2023-05</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>2023-06</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>2023-07</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>2023-08</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>2023-09</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>2023-10</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>2023-11</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>2023-12</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>2024-01</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>2024-02</t>
+        </is>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="AO3" t="inlineStr">
+        <is>
+          <t>2024-04</t>
+        </is>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>2024-05</t>
+        </is>
+      </c>
+      <c r="AQ3" t="inlineStr">
+        <is>
+          <t>2024-06</t>
+        </is>
+      </c>
+      <c r="AR3" t="inlineStr">
+        <is>
+          <t>2024-07</t>
+        </is>
+      </c>
+      <c r="AS3" t="inlineStr">
+        <is>
+          <t>2024-08</t>
+        </is>
+      </c>
+      <c r="AT3" t="inlineStr">
+        <is>
+          <t>2024-09</t>
+        </is>
+      </c>
+      <c r="AU3" t="inlineStr">
+        <is>
+          <t>2024-10</t>
+        </is>
+      </c>
+      <c r="AV3" t="inlineStr">
+        <is>
+          <t>2024-11</t>
+        </is>
+      </c>
+      <c r="AW3" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="AX3" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="AY3" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="AZ3" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="BA3" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="BB3" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="BC3" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="BD3" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="BE3" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="BF3" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="BG3" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="BH3" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="BI3" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>99.66687</v>
+      </c>
+      <c r="C4" t="n">
+        <v>99.80013</v>
+      </c>
+      <c r="D4" t="n">
+        <v>100.0481</v>
+      </c>
+      <c r="E4" t="n">
+        <v>100.2951</v>
+      </c>
+      <c r="F4" t="n">
+        <v>100.6629</v>
+      </c>
+      <c r="G4" t="n">
+        <v>100.9915</v>
+      </c>
+      <c r="H4" t="n">
+        <v>101.1128</v>
+      </c>
+      <c r="I4" t="n">
+        <v>101.1448</v>
+      </c>
+      <c r="J4" t="n">
+        <v>101.1952</v>
+      </c>
+      <c r="K4" t="n">
+        <v>101.0767</v>
+      </c>
+      <c r="L4" t="n">
+        <v>100.8589</v>
+      </c>
+      <c r="M4" t="n">
+        <v>100.6374</v>
+      </c>
+      <c r="N4" t="n">
+        <v>100.4013</v>
+      </c>
+      <c r="O4" t="n">
+        <v>99.86548999999999</v>
+      </c>
+      <c r="P4" t="n">
+        <v>98.99875</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>98.28712</v>
+      </c>
+      <c r="R4" t="n">
+        <v>97.83069999999999</v>
+      </c>
+      <c r="S4" t="n">
+        <v>97.43286000000001</v>
+      </c>
+      <c r="T4" t="n">
+        <v>97.01776</v>
+      </c>
+      <c r="U4" t="n">
+        <v>96.71699</v>
+      </c>
+      <c r="V4" t="n">
+        <v>96.46775</v>
+      </c>
+      <c r="W4" t="n">
+        <v>96.52760000000001</v>
+      </c>
+      <c r="X4" t="n">
+        <v>96.84836</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>97.28867</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>97.74052</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>98.13628</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>98.40537</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>98.68143000000001</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>98.83868</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>98.87727</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>98.84372999999999</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>98.75355</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>98.66359</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>98.60666000000001</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>98.58423999999999</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>98.64285</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>98.68248</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>98.88435</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>99.14597000000001</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>99.42401</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>99.58932</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>99.69349</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>99.76466000000001</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>99.72279</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>99.67807000000001</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>99.681</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>99.61151</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>99.54563</v>
+      </c>
+      <c r="AX4" t="n">
+        <v>99.47481999999999</v>
+      </c>
+      <c r="AY4" t="n">
+        <v>99.46912</v>
+      </c>
+      <c r="AZ4" t="n">
+        <v>99.53403</v>
+      </c>
+      <c r="BA4" t="n">
+        <v>99.61620000000001</v>
+      </c>
+      <c r="BB4" t="n">
+        <v>99.71351</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>99.75409999999999</v>
+      </c>
+      <c r="BD4" t="n">
+        <v>99.77131</v>
+      </c>
+      <c r="BE4" t="n">
+        <v>99.72692000000001</v>
+      </c>
+      <c r="BF4" t="n">
+        <v>99.68848</v>
+      </c>
+      <c r="BG4" t="n">
+        <v>99.58195000000001</v>
+      </c>
+      <c r="BH4" t="n">
+        <v>99.50239999999999</v>
+      </c>
+      <c r="BI4" t="n">
+        <v>99.52884</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>97.70017</v>
+      </c>
+      <c r="C5" t="n">
+        <v>98.22165</v>
+      </c>
+      <c r="D5" t="n">
+        <v>99.18996</v>
+      </c>
+      <c r="E5" t="n">
+        <v>99.98609</v>
+      </c>
+      <c r="F5" t="n">
+        <v>100.5841</v>
+      </c>
+      <c r="G5" t="n">
+        <v>100.9527</v>
+      </c>
+      <c r="H5" t="n">
+        <v>101.1354</v>
+      </c>
+      <c r="I5" t="n">
+        <v>101.1922</v>
+      </c>
+      <c r="J5" t="n">
+        <v>101.0743</v>
+      </c>
+      <c r="K5" t="n">
+        <v>100.764</v>
+      </c>
+      <c r="L5" t="n">
+        <v>100.1675</v>
+      </c>
+      <c r="M5" t="n">
+        <v>99.84808</v>
+      </c>
+      <c r="N5" t="n">
+        <v>99.56116</v>
+      </c>
+      <c r="O5" t="n">
+        <v>98.77092</v>
+      </c>
+      <c r="P5" t="n">
+        <v>97.1917</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>96.34094</v>
+      </c>
+      <c r="R5" t="n">
+        <v>95.89206</v>
+      </c>
+      <c r="S5" t="n">
+        <v>95.11839999999999</v>
+      </c>
+      <c r="T5" t="n">
+        <v>94.38748</v>
+      </c>
+      <c r="U5" t="n">
+        <v>94.29604</v>
+      </c>
+      <c r="V5" t="n">
+        <v>94.5082</v>
+      </c>
+      <c r="W5" t="n">
+        <v>95.00515</v>
+      </c>
+      <c r="X5" t="n">
+        <v>95.73175000000001</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>96.46687</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>97.029</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>97.30398</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>97.41732</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>97.79828999999999</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>98.30374</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>98.96724</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>99.35232000000001</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>99.04723</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>98.43823</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>98.13882</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>98.10148</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>98.22784</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>98.43429</v>
+      </c>
+      <c r="AM5" t="n">
+        <v>98.77981</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>99.14660000000001</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>99.43129</v>
+      </c>
+      <c r="AP5" t="n">
+        <v>99.57366</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>99.63921000000001</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>99.67677</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>99.70948</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>99.92326</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>100.1255</v>
+      </c>
+      <c r="AV5" t="n">
+        <v>100.3225</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>100.4038</v>
+      </c>
+      <c r="AX5" t="n">
+        <v>100.2281</v>
+      </c>
+      <c r="AY5" t="n">
+        <v>99.88108</v>
+      </c>
+      <c r="AZ5" t="n">
+        <v>99.51148999999999</v>
+      </c>
+      <c r="BA5" t="n">
+        <v>99.22671</v>
+      </c>
+      <c r="BB5" t="n">
+        <v>99.17956</v>
+      </c>
+      <c r="BC5" t="n">
+        <v>99.14695</v>
+      </c>
+      <c r="BD5" t="n">
+        <v>99.17019000000001</v>
+      </c>
+      <c r="BE5" t="n">
+        <v>99.41817</v>
+      </c>
+      <c r="BF5" t="n">
+        <v>99.74033</v>
+      </c>
+      <c r="BG5" t="n">
+        <v>99.92717</v>
+      </c>
+      <c r="BH5" t="n">
+        <v>99.89664</v>
+      </c>
+      <c r="BI5" t="n">
+        <v>99.76157000000001</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>98.85334</v>
+      </c>
+      <c r="C6" t="n">
+        <v>99.05428000000001</v>
+      </c>
+      <c r="D6" t="n">
+        <v>99.56672</v>
+      </c>
+      <c r="E6" t="n">
+        <v>100.1922</v>
+      </c>
+      <c r="F6" t="n">
+        <v>100.9601</v>
+      </c>
+      <c r="G6" t="n">
+        <v>101.5277</v>
+      </c>
+      <c r="H6" t="n">
+        <v>101.516</v>
+      </c>
+      <c r="I6" t="n">
+        <v>101.277</v>
+      </c>
+      <c r="J6" t="n">
+        <v>101.1606</v>
+      </c>
+      <c r="K6" t="n">
+        <v>100.8813</v>
+      </c>
+      <c r="L6" t="n">
+        <v>100.5841</v>
+      </c>
+      <c r="M6" t="n">
+        <v>100.2511</v>
+      </c>
+      <c r="N6" t="n">
+        <v>99.81926</v>
+      </c>
+      <c r="O6" t="n">
+        <v>99.10256</v>
+      </c>
+      <c r="P6" t="n">
+        <v>97.99290000000001</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>97.40778</v>
+      </c>
+      <c r="R6" t="n">
+        <v>97.14031</v>
+      </c>
+      <c r="S6" t="n">
+        <v>96.95766</v>
+      </c>
+      <c r="T6" t="n">
+        <v>96.91983999999999</v>
+      </c>
+      <c r="U6" t="n">
+        <v>96.99772</v>
+      </c>
+      <c r="V6" t="n">
+        <v>96.95685</v>
+      </c>
+      <c r="W6" t="n">
+        <v>97.04956</v>
+      </c>
+      <c r="X6" t="n">
+        <v>97.1575</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>97.08394</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>96.98483</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>96.95466999999999</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>97.12567</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>97.49252</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>97.94678</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>98.34627</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>98.52292</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>98.47356000000001</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>98.36293000000001</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>98.39339</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>98.6589</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>98.88348000000001</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>98.97713</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>98.83687999999999</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>98.71513</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>98.5899</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>98.59456</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>98.6041</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>98.69248</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>98.9177</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>99.02813</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>98.85326000000001</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>98.52699</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>98.35442</v>
+      </c>
+      <c r="AX6" t="n">
+        <v>98.52218999999999</v>
+      </c>
+      <c r="AY6" t="n">
+        <v>98.62938</v>
+      </c>
+      <c r="AZ6" t="n">
+        <v>98.46934</v>
+      </c>
+      <c r="BA6" t="n">
+        <v>98.17923</v>
+      </c>
+      <c r="BB6" t="n">
+        <v>97.93805999999999</v>
+      </c>
+      <c r="BC6" t="n">
+        <v>97.82043</v>
+      </c>
+      <c r="BD6" t="n">
+        <v>97.75543</v>
+      </c>
+      <c r="BE6" t="n">
+        <v>97.66985</v>
+      </c>
+      <c r="BF6" t="n">
+        <v>97.73289</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>98.00545</v>
+      </c>
+      <c r="BH6" t="n">
+        <v>98.17167999999999</v>
+      </c>
+      <c r="BI6" t="n">
+        <v>98.24182</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>gdp_current_prices</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>geo</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2016</v>
+      </c>
+      <c r="C12" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2018</v>
+      </c>
+      <c r="E12" t="n">
+        <v>2019</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H12" t="n">
+        <v>2022</v>
+      </c>
+      <c r="I12" t="n">
+        <v>2023</v>
+      </c>
+      <c r="J12" t="n">
+        <v>2024</v>
+      </c>
+      <c r="K12" t="n">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>DEU</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>3535.812</v>
+      </c>
+      <c r="C13" t="n">
+        <v>3764.023</v>
+      </c>
+      <c r="D13" t="n">
+        <v>4057.272</v>
+      </c>
+      <c r="E13" t="n">
+        <v>3960.332</v>
+      </c>
+      <c r="F13" t="n">
+        <v>3938.244</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4358.147</v>
+      </c>
+      <c r="H13" t="n">
+        <v>4204.327</v>
+      </c>
+      <c r="I13" t="n">
+        <v>4563.523</v>
+      </c>
+      <c r="J13" t="n">
+        <v>4684.182</v>
+      </c>
+      <c r="K13" t="n">
+        <v>5013.574</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ESP</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1242.673</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1321.288</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1432.292</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1403.651</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1288.751</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1462.216</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1449.99</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1619.949</v>
+      </c>
+      <c r="J14" t="n">
+        <v>1725.152</v>
+      </c>
+      <c r="K14" t="n">
+        <v>1891.371</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2469.726</v>
+      </c>
+      <c r="C15" t="n">
+        <v>2587.955</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2782.838</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2723.094</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2645.806</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2968.405</v>
+      </c>
+      <c r="H15" t="n">
+        <v>2796.987</v>
+      </c>
+      <c r="I15" t="n">
+        <v>3061.093</v>
+      </c>
+      <c r="J15" t="n">
+        <v>3160.902</v>
+      </c>
+      <c r="K15" t="n">
+        <v>3361.557</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>gdp_per_capita_current_prices</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>geo</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2016</v>
+      </c>
+      <c r="C21" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2018</v>
+      </c>
+      <c r="E21" t="n">
+        <v>2019</v>
+      </c>
+      <c r="F21" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G21" t="n">
+        <v>2021</v>
+      </c>
+      <c r="H21" t="n">
+        <v>2022</v>
+      </c>
+      <c r="I21" t="n">
+        <v>2023</v>
+      </c>
+      <c r="J21" t="n">
+        <v>2024</v>
+      </c>
+      <c r="K21" t="n">
+        <v>2025</v>
+      </c>
+      <c r="L21" t="n">
+        <v>2026</v>
+      </c>
+      <c r="M21" t="n">
+        <v>2027</v>
+      </c>
+      <c r="N21" t="n">
+        <v>2028</v>
+      </c>
+      <c r="O21" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P21" t="n">
+        <v>2030</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>DEU</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>43189.577</v>
+      </c>
+      <c r="C22" t="n">
+        <v>45881.456</v>
+      </c>
+      <c r="D22" t="n">
+        <v>49384.527</v>
+      </c>
+      <c r="E22" t="n">
+        <v>48177.607</v>
+      </c>
+      <c r="F22" t="n">
+        <v>47953.683</v>
+      </c>
+      <c r="G22" t="n">
+        <v>53151.541</v>
+      </c>
+      <c r="H22" t="n">
+        <v>50943.628</v>
+      </c>
+      <c r="I22" t="n">
+        <v>54793.074</v>
+      </c>
+      <c r="J22" t="n">
+        <v>56086.903</v>
+      </c>
+      <c r="K22" t="n">
+        <v>59925.317</v>
+      </c>
+      <c r="L22" t="n">
+        <v>63599.502</v>
+      </c>
+      <c r="M22" t="n">
+        <v>65580.908</v>
+      </c>
+      <c r="N22" t="n">
+        <v>67653.54300000001</v>
+      </c>
+      <c r="O22" t="n">
+        <v>69713.379</v>
+      </c>
+      <c r="P22" t="n">
+        <v>71683.47500000001</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ESP</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>26725.642</v>
+      </c>
+      <c r="C23" t="n">
+        <v>28326.416</v>
+      </c>
+      <c r="D23" t="n">
+        <v>30526.94</v>
+      </c>
+      <c r="E23" t="n">
+        <v>29664.183</v>
+      </c>
+      <c r="F23" t="n">
+        <v>27188.392</v>
+      </c>
+      <c r="G23" t="n">
+        <v>30792.106</v>
+      </c>
+      <c r="H23" t="n">
+        <v>30154.509</v>
+      </c>
+      <c r="I23" t="n">
+        <v>33312.918</v>
+      </c>
+      <c r="J23" t="n">
+        <v>35151.242</v>
+      </c>
+      <c r="K23" t="n">
+        <v>38039.876</v>
+      </c>
+      <c r="L23" t="n">
+        <v>40581.506</v>
+      </c>
+      <c r="M23" t="n">
+        <v>41888.427</v>
+      </c>
+      <c r="N23" t="n">
+        <v>43059.815</v>
+      </c>
+      <c r="O23" t="n">
+        <v>44363.981</v>
+      </c>
+      <c r="P23" t="n">
+        <v>45765.843</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>37081.496</v>
+      </c>
+      <c r="C24" t="n">
+        <v>38756.651</v>
+      </c>
+      <c r="D24" t="n">
+        <v>41539.756</v>
+      </c>
+      <c r="E24" t="n">
+        <v>40487.302</v>
+      </c>
+      <c r="F24" t="n">
+        <v>39230.928</v>
+      </c>
+      <c r="G24" t="n">
+        <v>43848.345</v>
+      </c>
+      <c r="H24" t="n">
+        <v>41095.77</v>
+      </c>
+      <c r="I24" t="n">
+        <v>44853.761</v>
+      </c>
+      <c r="J24" t="n">
+        <v>46187.295</v>
+      </c>
+      <c r="K24" t="n">
+        <v>48981.965</v>
+      </c>
+      <c r="L24" t="n">
+        <v>51707.603</v>
+      </c>
+      <c r="M24" t="n">
+        <v>53048.574</v>
+      </c>
+      <c r="N24" t="n">
+        <v>54515.019</v>
+      </c>
+      <c r="O24" t="n">
+        <v>56050.844</v>
+      </c>
+      <c r="P24" t="n">
+        <v>57606.464</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>inflation_average_consumer_prices</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>geo</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C30" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D30" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E30" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F30" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G30" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H30" t="n">
+        <v>2027</v>
+      </c>
+      <c r="I30" t="n">
+        <v>2028</v>
+      </c>
+      <c r="J30" t="n">
+        <v>2029</v>
+      </c>
+      <c r="K30" t="n">
+        <v>2030</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>DEU</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="C31" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="D31" t="n">
+        <v>3</v>
+      </c>
+      <c r="E31" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="G31" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H31" t="n">
+        <v>2</v>
+      </c>
+      <c r="I31" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="J31" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="K31" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ESP</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="C32" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="D32" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="E32" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F32" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G32" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H32" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I32" t="n">
+        <v>2</v>
+      </c>
+      <c r="J32" t="n">
+        <v>2</v>
+      </c>
+      <c r="K32" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="C33" t="n">
+        <v>7</v>
+      </c>
+      <c r="D33" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E33" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G33" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H33" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I33" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J33" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>population</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>geo</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C39" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D39" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E39" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F39" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G39" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H39" t="n">
+        <v>2027</v>
+      </c>
+      <c r="I39" t="n">
+        <v>2028</v>
+      </c>
+      <c r="J39" t="n">
+        <v>2029</v>
+      </c>
+      <c r="K39" t="n">
+        <v>2030</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>DEU</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>81.995</v>
+      </c>
+      <c r="C40" t="n">
+        <v>82.529</v>
+      </c>
+      <c r="D40" t="n">
+        <v>83.28700000000001</v>
+      </c>
+      <c r="E40" t="n">
+        <v>83.517</v>
+      </c>
+      <c r="F40" t="n">
+        <v>83.664</v>
+      </c>
+      <c r="G40" t="n">
+        <v>83.777</v>
+      </c>
+      <c r="H40" t="n">
+        <v>83.845</v>
+      </c>
+      <c r="I40" t="n">
+        <v>83.874</v>
+      </c>
+      <c r="J40" t="n">
+        <v>83.89100000000001</v>
+      </c>
+      <c r="K40" t="n">
+        <v>83.893</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>ESP</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>47.487</v>
+      </c>
+      <c r="C41" t="n">
+        <v>48.085</v>
+      </c>
+      <c r="D41" t="n">
+        <v>48.628</v>
+      </c>
+      <c r="E41" t="n">
+        <v>49.078</v>
+      </c>
+      <c r="F41" t="n">
+        <v>49.721</v>
+      </c>
+      <c r="G41" t="n">
+        <v>50.314</v>
+      </c>
+      <c r="H41" t="n">
+        <v>50.84</v>
+      </c>
+      <c r="I41" t="n">
+        <v>51.294</v>
+      </c>
+      <c r="J41" t="n">
+        <v>51.679</v>
+      </c>
+      <c r="K41" t="n">
+        <v>52.004</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>67.697</v>
+      </c>
+      <c r="C42" t="n">
+        <v>68.06</v>
+      </c>
+      <c r="D42" t="n">
+        <v>68.246</v>
+      </c>
+      <c r="E42" t="n">
+        <v>68.437</v>
+      </c>
+      <c r="F42" t="n">
+        <v>68.628</v>
+      </c>
+      <c r="G42" t="n">
+        <v>68.821</v>
+      </c>
+      <c r="H42" t="n">
+        <v>69.014</v>
+      </c>
+      <c r="I42" t="n">
+        <v>69.20699999999999</v>
+      </c>
+      <c r="J42" t="n">
+        <v>69.401</v>
+      </c>
+      <c r="K42" t="n">
+        <v>69.596</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>real_gdp_growth_percent</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>geo</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C48" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D48" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E48" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F48" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G48" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H48" t="n">
+        <v>2027</v>
+      </c>
+      <c r="I48" t="n">
+        <v>2028</v>
+      </c>
+      <c r="J48" t="n">
+        <v>2029</v>
+      </c>
+      <c r="K48" t="n">
+        <v>2030</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>DEU</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D49" t="n">
+        <v>-0.9</v>
+      </c>
+      <c r="E49" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H49" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I49" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="J49" t="n">
+        <v>1</v>
+      </c>
+      <c r="K49" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>ESP</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="C50" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="D50" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E50" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F50" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="G50" t="n">
+        <v>2</v>
+      </c>
+      <c r="H50" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="I50" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J50" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="K50" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="C51" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="D51" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E51" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H51" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="I51" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="J51" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="K51" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>unemployment_rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>geo</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C57" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D57" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E57" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F57" t="n">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>DEU</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="C58" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="D58" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="E58" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F58" t="n">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>ESP</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="C59" t="n">
+        <v>13</v>
+      </c>
+      <c r="D59" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="E59" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="F59" t="n">
+        <v>10.8</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="C60" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="D60" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="E60" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="F60" t="n">
+        <v>7.6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>